<commit_message>
Update mechanism of action through stimulus in bcio_moa.xlsx
</commit_message>
<xml_diff>
--- a/MechanismOfAction/bcio_moa.xlsx
+++ b/MechanismOfAction/bcio_moa.xlsx
@@ -751,7 +751,7 @@
         </is>
       </c>
       <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
+      <c r="F5" s="3" t="inlineStr"/>
       <c r="G5" s="3" t="n"/>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="inlineStr">
@@ -15980,7 +15980,7 @@
       </c>
       <c r="L260" s="3" t="n"/>
       <c r="M260" s="3" t="n"/>
-      <c r="N260" s="3" t="n"/>
+      <c r="N260" s="3" t="inlineStr"/>
       <c r="O260" s="3" t="n"/>
       <c r="P260" s="3" t="n"/>
       <c r="Q260" s="3" t="n"/>
@@ -23640,7 +23640,7 @@
         </is>
       </c>
       <c r="E389" s="3" t="n"/>
-      <c r="F389" s="3" t="n"/>
+      <c r="F389" s="3" t="inlineStr"/>
       <c r="G389" s="3" t="n"/>
       <c r="H389" s="3" t="n"/>
       <c r="I389" s="3" t="n"/>
@@ -23654,7 +23654,7 @@
       <c r="K389" s="3" t="n"/>
       <c r="L389" s="3" t="inlineStr">
         <is>
-          <t>stimulus</t>
+          <t>stimulus; behavioural cue; external stimulus; reminder stimulus; extrinsic reward; internal stimulus; internal stimulus for behaviour; mental stimulus for behaviour; intrinsic reward</t>
         </is>
       </c>
       <c r="M389" s="3" t="n"/>
@@ -27698,32 +27698,32 @@
           <t>self-efficacy belief</t>
         </is>
       </c>
-      <c r="E458" s="4" t="inlineStr"/>
-      <c r="F458" s="4" t="inlineStr"/>
-      <c r="G458" s="4" t="inlineStr"/>
-      <c r="H458" s="4" t="inlineStr"/>
-      <c r="I458" s="4" t="inlineStr"/>
-      <c r="J458" s="4" t="inlineStr"/>
-      <c r="K458" s="4" t="inlineStr"/>
-      <c r="L458" s="4" t="inlineStr"/>
-      <c r="M458" s="4" t="inlineStr"/>
-      <c r="N458" s="4" t="inlineStr"/>
-      <c r="O458" s="4" t="inlineStr"/>
-      <c r="P458" s="4" t="inlineStr"/>
-      <c r="Q458" s="4" t="inlineStr"/>
-      <c r="R458" s="4" t="inlineStr"/>
+      <c r="E458" s="4" t="n"/>
+      <c r="F458" s="4" t="n"/>
+      <c r="G458" s="4" t="n"/>
+      <c r="H458" s="4" t="n"/>
+      <c r="I458" s="4" t="n"/>
+      <c r="J458" s="4" t="n"/>
+      <c r="K458" s="4" t="n"/>
+      <c r="L458" s="4" t="n"/>
+      <c r="M458" s="4" t="n"/>
+      <c r="N458" s="4" t="n"/>
+      <c r="O458" s="4" t="n"/>
+      <c r="P458" s="4" t="n"/>
+      <c r="Q458" s="4" t="n"/>
+      <c r="R458" s="4" t="n"/>
       <c r="S458" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="T458" s="4" t="inlineStr"/>
-      <c r="U458" s="4" t="inlineStr"/>
-      <c r="V458" s="4" t="inlineStr"/>
+      <c r="T458" s="4" t="n"/>
+      <c r="U458" s="4" t="n"/>
+      <c r="V458" s="4" t="n"/>
       <c r="W458" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="X458" s="4" t="inlineStr"/>
+      <c r="X458" s="4" t="n"/>
     </row>
     <row r="459">
       <c r="A459" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Update mechanism of action through cognitive representation in bcio_moa.xlsx
</commit_message>
<xml_diff>
--- a/MechanismOfAction/bcio_moa.xlsx
+++ b/MechanismOfAction/bcio_moa.xlsx
@@ -23126,7 +23126,7 @@
         </is>
       </c>
       <c r="E381" s="3" t="n"/>
-      <c r="F381" s="3" t="n"/>
+      <c r="F381" s="3" t="inlineStr"/>
       <c r="G381" s="3" t="n"/>
       <c r="H381" s="3" t="n"/>
       <c r="I381" s="3" t="n"/>
@@ -23144,7 +23144,7 @@
       </c>
       <c r="L381" s="3" t="inlineStr">
         <is>
-          <t>cognitive representation</t>
+          <t>cognitive representation; cognitive representation of one’s behaviour; cognitive representation of an alternative behaviour	; goal; well-specified goal; self-initiated goal; assigned goal; learning goal; active goal; accepted assigned goal; goal about one’s resources; proximal goal; hedonic goal; behavioural goal; normative goal; collaborative goal; distal goal; background goal; desired standard; desired standard for self-identity; desired self-regulatory standard; social representation of a behaviour; propositional cognitive representation; identity; group identity; self-identity; professional identity; social identity	; similarity to other people; affective appraisal; behavioural consequence appraisal process; social consequence of behaviour appraisal process; appraisal of goal importance; appraisal of expectedness; appraisal of desirability; appraisal of desirability of consequences; appraisal of obligation to act; appraisal of immediacy; appraisal of pleasantness; appraisal of dangerousness; affective appraisal of possible consequences; self-identity appraisal process; self-identity appraisal informed by one’s behaviour; appraisal of social identity; appraisal of causal agency; appraisal as caused by external non-human factors; appraisal as caused by an other; appraisal as caused by self; appraisal of avoidability of consequences; comparative desirability appraisal; mental image</t>
         </is>
       </c>
       <c r="M381" s="3" t="n"/>
@@ -23193,7 +23193,7 @@
           <t>behaviour change intervention mechanism of action</t>
         </is>
       </c>
-      <c r="E382" s="3" t="inlineStr"/>
+      <c r="E382" s="3" t="n"/>
       <c r="F382" s="3" t="n"/>
       <c r="G382" s="3" t="n"/>
       <c r="H382" s="3" t="n"/>
@@ -23536,7 +23536,7 @@
       </c>
       <c r="L387" s="3" t="n"/>
       <c r="M387" s="3" t="n"/>
-      <c r="N387" s="3" t="inlineStr"/>
+      <c r="N387" s="3" t="n"/>
       <c r="O387" s="3" t="n"/>
       <c r="P387" s="3" t="n"/>
       <c r="Q387" s="3" t="n"/>
@@ -23655,7 +23655,7 @@
 In this definition, ‘change’ refers to change from what would have been the case rather than change from an existing state of affairs. This is to capture the fact that mechanisms of action can act to sustain a current state of affairs, for example preventing smoking uptake. In the definition, ‘some change’ captures changes in salience, change in valence, or being added, increased, decreased, manifested/realised, created, started, stopped or altered rate.</t>
         </is>
       </c>
-      <c r="K389" s="3" t="inlineStr"/>
+      <c r="K389" s="3" t="n"/>
       <c r="L389" s="3" t="inlineStr">
         <is>
           <t>stimulus; behavioural cue; external stimulus; reminder stimulus; extrinsic reward; internal stimulus; internal stimulus for behaviour; mental stimulus for behaviour; intrinsic reward</t>

</xml_diff>